<commit_message>
Finalize pre-production version and generate gerbers
</commit_message>
<xml_diff>
--- a/Project Outputs for TSI_SAMP_SAMI_V3.4/Generate Files/BOM/Bill of Materials-TSI_SAMP_SAMI_V3.4(SAMI_V3.5).xlsx
+++ b/Project Outputs for TSI_SAMP_SAMI_V3.4/Generate Files/BOM/Bill of Materials-TSI_SAMP_SAMI_V3.4(SAMI_V3.5).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\biark\Documents\CanAssist\TSI_SAMP_SAMI\Project Outputs for TSI_SAMP_SAMI_V3.4\Generate Files\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E32609E0-5D4D-46CF-9F65-FF579AD1D728}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{70EDD994-359F-49BC-9BB6-0B2FFBDCEF49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{B1B3122D-2FDA-4FE2-AC69-5DB844443518}"/>
+    <workbookView xWindow="2280" yWindow="2280" windowWidth="19200" windowHeight="11170" xr2:uid="{B0082170-DDA8-4935-AA34-F41290B8C798}"/>
   </bookViews>
   <sheets>
     <sheet name="Bill of Materials-TSI_SAMP_SAMI" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="716" uniqueCount="390">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="716" uniqueCount="389">
   <si>
     <t>Revision ID</t>
   </si>
@@ -149,7 +149,7 @@
     <t>Yageo - CC0603MRX5R7BB106 - CAP, MLCC, X5R, 10uF, 16V, 0603</t>
   </si>
   <si>
-    <t>C9, C12, C15, C21, C25, C35, C38, C39, C63, C67, C68</t>
+    <t>C9, C12, C15, C21, C25, C35, C38, C39, C63, C67, C68, C69</t>
   </si>
   <si>
     <t>CC0603MRX5R7BB106</t>
@@ -542,7 +542,7 @@
     <t>SJ-3566AN</t>
   </si>
   <si>
-    <t>CP-SJ-3566AN-ND</t>
+    <t>490-SJ-3566AN</t>
   </si>
   <si>
     <t>3.5mm DBL</t>
@@ -740,7 +740,7 @@
     <t>RC0603JR-072ML</t>
   </si>
   <si>
-    <t>311-2.0MGRCT-ND</t>
+    <t>603-RC0603JR-072ML</t>
   </si>
   <si>
     <t>20K</t>
@@ -770,7 +770,7 @@
     <t>RC0603FR-072K1L</t>
   </si>
   <si>
-    <t>311-2.10KHRCT-ND</t>
+    <t>603-RC0603FR-072K1L</t>
   </si>
   <si>
     <t>10k</t>
@@ -1022,7 +1022,7 @@
     <t>MAX9744ETH+T</t>
   </si>
   <si>
-    <t>700-MAX9744ETH+T</t>
+    <t>MAX9744ETH+TCT-ND</t>
   </si>
   <si>
     <t>MAX6818EAP+T</t>
@@ -1112,10 +1112,7 @@
     <t>1681</t>
   </si>
   <si>
-    <t>Digi-Key</t>
-  </si>
-  <si>
-    <t>1528-2645-ND</t>
+    <t>485-1681</t>
   </si>
   <si>
     <t>IC BUF ESD</t>
@@ -1604,7 +1601,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6055CE56-921C-4CD6-986A-28DE460B4D5B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA7B93E9-26FE-4C90-941D-E8DAC8A59544}">
   <dimension ref="A1:Q65"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1726,7 +1723,7 @@
         <v>0.34</v>
       </c>
       <c r="Q2" s="1">
-        <v>278801</v>
+        <v>248879</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.35">
@@ -1775,7 +1772,7 @@
         <v>0.45</v>
       </c>
       <c r="Q3" s="1">
-        <v>801</v>
+        <v>391</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.35">
@@ -1797,7 +1794,7 @@
       </c>
       <c r="G4" s="1"/>
       <c r="H4" s="1">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I4" s="2" t="s">
         <v>22</v>
@@ -1821,10 +1818,10 @@
         <v>0.17499999999999999</v>
       </c>
       <c r="P4" s="1">
-        <v>1.93</v>
+        <v>2.1</v>
       </c>
       <c r="Q4" s="1">
-        <v>6877</v>
+        <v>17717</v>
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.35">
@@ -1873,7 +1870,7 @@
         <v>0.13</v>
       </c>
       <c r="Q5" s="1">
-        <v>22730</v>
+        <v>22350</v>
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.35">
@@ -1922,7 +1919,7 @@
         <v>0.23</v>
       </c>
       <c r="Q6" s="1">
-        <v>659271</v>
+        <v>546364</v>
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.35">
@@ -1971,7 +1968,7 @@
         <v>0.36</v>
       </c>
       <c r="Q7" s="1">
-        <v>383282</v>
+        <v>366595</v>
       </c>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.35">
@@ -2020,7 +2017,7 @@
         <v>1.94</v>
       </c>
       <c r="Q8" s="1">
-        <v>16230</v>
+        <v>16225</v>
       </c>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.35">
@@ -2069,7 +2066,7 @@
         <v>0.24</v>
       </c>
       <c r="Q9" s="1">
-        <v>93757</v>
+        <v>89087</v>
       </c>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.35">
@@ -2118,7 +2115,7 @@
         <v>0.66</v>
       </c>
       <c r="Q10" s="1">
-        <v>227181</v>
+        <v>225070</v>
       </c>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.35">
@@ -2167,7 +2164,7 @@
         <v>0.36</v>
       </c>
       <c r="Q11" s="1">
-        <v>31656</v>
+        <v>30423</v>
       </c>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.35">
@@ -2216,7 +2213,7 @@
         <v>0.32</v>
       </c>
       <c r="Q12" s="1">
-        <v>1511</v>
+        <v>1441</v>
       </c>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.35">
@@ -2265,7 +2262,7 @@
         <v>0.2</v>
       </c>
       <c r="Q13" s="1">
-        <v>32875</v>
+        <v>28107</v>
       </c>
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.35">
@@ -2314,7 +2311,7 @@
         <v>0.7</v>
       </c>
       <c r="Q14" s="1">
-        <v>35180</v>
+        <v>52423</v>
       </c>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.35">
@@ -2363,7 +2360,7 @@
         <v>0.1</v>
       </c>
       <c r="Q15" s="1">
-        <v>687016</v>
+        <v>678834</v>
       </c>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.35">
@@ -2455,13 +2452,13 @@
         <v>110</v>
       </c>
       <c r="O17" s="1">
-        <v>1.4</v>
+        <v>1.58</v>
       </c>
       <c r="P17" s="1">
-        <v>2.8</v>
+        <v>3.16</v>
       </c>
       <c r="Q17" s="1">
-        <v>16773</v>
+        <v>20394</v>
       </c>
     </row>
     <row r="18" spans="1:17" x14ac:dyDescent="0.35">
@@ -2510,7 +2507,7 @@
         <v>0.39</v>
       </c>
       <c r="Q18" s="1">
-        <v>34626</v>
+        <v>28281</v>
       </c>
     </row>
     <row r="19" spans="1:17" x14ac:dyDescent="0.35">
@@ -2559,7 +2556,7 @@
         <v>0.15</v>
       </c>
       <c r="Q19" s="1">
-        <v>1552439</v>
+        <v>1321305</v>
       </c>
     </row>
     <row r="20" spans="1:17" x14ac:dyDescent="0.35">
@@ -2608,7 +2605,7 @@
         <v>0.3</v>
       </c>
       <c r="Q20" s="1">
-        <v>410475</v>
+        <v>386999</v>
       </c>
     </row>
     <row r="21" spans="1:17" x14ac:dyDescent="0.35">
@@ -2657,7 +2654,7 @@
         <v>35.450000000000003</v>
       </c>
       <c r="Q21" s="1">
-        <v>103</v>
+        <v>142</v>
       </c>
     </row>
     <row r="22" spans="1:17" x14ac:dyDescent="0.35">
@@ -2706,7 +2703,7 @@
         <v>0.87</v>
       </c>
       <c r="Q22" s="1">
-        <v>55351</v>
+        <v>53673</v>
       </c>
     </row>
     <row r="23" spans="1:17" x14ac:dyDescent="0.35">
@@ -2755,7 +2752,7 @@
         <v>0.4</v>
       </c>
       <c r="Q23" s="1">
-        <v>59155</v>
+        <v>50115</v>
       </c>
     </row>
     <row r="24" spans="1:17" x14ac:dyDescent="0.35">
@@ -2804,7 +2801,7 @@
         <v>43.71</v>
       </c>
       <c r="Q24" s="1">
-        <v>1848</v>
+        <v>2009</v>
       </c>
     </row>
     <row r="25" spans="1:17" x14ac:dyDescent="0.35">
@@ -2853,7 +2850,7 @@
         <v>0.83</v>
       </c>
       <c r="Q25" s="1">
-        <v>8348</v>
+        <v>8212</v>
       </c>
     </row>
     <row r="26" spans="1:17" x14ac:dyDescent="0.35">
@@ -2890,19 +2887,19 @@
         <v>25</v>
       </c>
       <c r="M26" s="2" t="s">
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="N26" s="2" t="s">
         <v>167</v>
       </c>
       <c r="O26" s="1">
-        <v>1.79</v>
+        <v>1.69</v>
       </c>
       <c r="P26" s="1">
-        <v>5.37</v>
+        <v>5.07</v>
       </c>
       <c r="Q26" s="1">
-        <v>193</v>
+        <v>94</v>
       </c>
     </row>
     <row r="27" spans="1:17" x14ac:dyDescent="0.35">
@@ -2951,7 +2948,7 @@
         <v>3.62</v>
       </c>
       <c r="Q27" s="1">
-        <v>30810</v>
+        <v>29500</v>
       </c>
     </row>
     <row r="28" spans="1:17" x14ac:dyDescent="0.35">
@@ -3000,7 +2997,7 @@
         <v>3.62</v>
       </c>
       <c r="Q28" s="1">
-        <v>30810</v>
+        <v>29500</v>
       </c>
     </row>
     <row r="29" spans="1:17" x14ac:dyDescent="0.35">
@@ -3049,7 +3046,7 @@
         <v>4.43</v>
       </c>
       <c r="Q29" s="1">
-        <v>31179</v>
+        <v>36612</v>
       </c>
     </row>
     <row r="30" spans="1:17" x14ac:dyDescent="0.35">
@@ -3147,7 +3144,7 @@
         <v>0.81</v>
       </c>
       <c r="Q31" s="1">
-        <v>208226</v>
+        <v>216932</v>
       </c>
     </row>
     <row r="32" spans="1:17" x14ac:dyDescent="0.35">
@@ -3196,7 +3193,7 @@
         <v>2.78</v>
       </c>
       <c r="Q32" s="1">
-        <v>5062</v>
+        <v>4822</v>
       </c>
     </row>
     <row r="33" spans="1:17" x14ac:dyDescent="0.35">
@@ -3245,7 +3242,7 @@
         <v>1.4</v>
       </c>
       <c r="Q33" s="1">
-        <v>15802</v>
+        <v>15307</v>
       </c>
     </row>
     <row r="34" spans="1:17" x14ac:dyDescent="0.35">
@@ -3294,7 +3291,7 @@
         <v>0.49</v>
       </c>
       <c r="Q34" s="1">
-        <v>4715</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="35" spans="1:17" x14ac:dyDescent="0.35">
@@ -3343,7 +3340,7 @@
         <v>0.48</v>
       </c>
       <c r="Q35" s="1">
-        <v>108533</v>
+        <v>104482</v>
       </c>
     </row>
     <row r="36" spans="1:17" x14ac:dyDescent="0.35">
@@ -3392,7 +3389,7 @@
         <v>0.69</v>
       </c>
       <c r="Q36" s="1">
-        <v>105838</v>
+        <v>105743</v>
       </c>
     </row>
     <row r="37" spans="1:17" x14ac:dyDescent="0.35">
@@ -3478,7 +3475,7 @@
         <v>25</v>
       </c>
       <c r="M38" s="2" t="s">
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="N38" s="2" t="s">
         <v>233</v>
@@ -3490,7 +3487,7 @@
         <v>0.1</v>
       </c>
       <c r="Q38" s="1">
-        <v>45906</v>
+        <v>40267</v>
       </c>
     </row>
     <row r="39" spans="1:17" x14ac:dyDescent="0.35">
@@ -3539,7 +3536,7 @@
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="Q39" s="1">
-        <v>2774839</v>
+        <v>2710093</v>
       </c>
     </row>
     <row r="40" spans="1:17" x14ac:dyDescent="0.35">
@@ -3576,7 +3573,7 @@
         <v>25</v>
       </c>
       <c r="M40" s="2" t="s">
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="N40" s="2" t="s">
         <v>243</v>
@@ -3588,7 +3585,7 @@
         <v>0.1</v>
       </c>
       <c r="Q40" s="1">
-        <v>61862</v>
+        <v>58506</v>
       </c>
     </row>
     <row r="41" spans="1:17" x14ac:dyDescent="0.35">
@@ -3637,7 +3634,7 @@
         <v>0.18</v>
       </c>
       <c r="Q41" s="1">
-        <v>3294268</v>
+        <v>6562551</v>
       </c>
     </row>
     <row r="42" spans="1:17" x14ac:dyDescent="0.35">
@@ -3686,7 +3683,7 @@
         <v>0.2</v>
       </c>
       <c r="Q42" s="1">
-        <v>62310</v>
+        <v>62060</v>
       </c>
     </row>
     <row r="43" spans="1:17" x14ac:dyDescent="0.35">
@@ -3735,7 +3732,7 @@
         <v>0.28999999999999998</v>
       </c>
       <c r="Q43" s="1">
-        <v>589223</v>
+        <v>571540</v>
       </c>
     </row>
     <row r="44" spans="1:17" x14ac:dyDescent="0.35">
@@ -3784,7 +3781,7 @@
         <v>0.31680000000000003</v>
       </c>
       <c r="Q44" s="1">
-        <v>15175</v>
+        <v>80639</v>
       </c>
     </row>
     <row r="45" spans="1:17" x14ac:dyDescent="0.35">
@@ -3827,13 +3824,13 @@
         <v>269</v>
       </c>
       <c r="O45" s="1">
-        <v>0.16</v>
+        <v>0.17</v>
       </c>
       <c r="P45" s="1">
-        <v>0.32</v>
+        <v>0.34</v>
       </c>
       <c r="Q45" s="1">
-        <v>125704</v>
+        <v>125657</v>
       </c>
     </row>
     <row r="46" spans="1:17" x14ac:dyDescent="0.35">
@@ -3882,7 +3879,7 @@
         <v>0.09</v>
       </c>
       <c r="Q46" s="1">
-        <v>97743</v>
+        <v>96583</v>
       </c>
     </row>
     <row r="47" spans="1:17" x14ac:dyDescent="0.35">
@@ -3925,13 +3922,13 @@
         <v>279</v>
       </c>
       <c r="O47" s="1">
-        <v>0.16</v>
+        <v>0.17</v>
       </c>
       <c r="P47" s="1">
-        <v>0.16</v>
+        <v>0.17</v>
       </c>
       <c r="Q47" s="1">
-        <v>20048</v>
+        <v>20017</v>
       </c>
     </row>
     <row r="48" spans="1:17" x14ac:dyDescent="0.35">
@@ -3980,7 +3977,7 @@
         <v>0.1</v>
       </c>
       <c r="Q48" s="1">
-        <v>1125442</v>
+        <v>1845030</v>
       </c>
     </row>
     <row r="49" spans="1:17" x14ac:dyDescent="0.35">
@@ -4029,7 +4026,7 @@
         <v>0.32</v>
       </c>
       <c r="Q49" s="1">
-        <v>22190</v>
+        <v>22140</v>
       </c>
     </row>
     <row r="50" spans="1:17" x14ac:dyDescent="0.35">
@@ -4078,7 +4075,7 @@
         <v>0.72</v>
       </c>
       <c r="Q50" s="1">
-        <v>302</v>
+        <v>4220</v>
       </c>
     </row>
     <row r="51" spans="1:17" x14ac:dyDescent="0.35">
@@ -4127,7 +4124,7 @@
         <v>5</v>
       </c>
       <c r="Q51" s="1">
-        <v>6319</v>
+        <v>6213</v>
       </c>
     </row>
     <row r="52" spans="1:17" x14ac:dyDescent="0.35">
@@ -4176,7 +4173,7 @@
         <v>0.26</v>
       </c>
       <c r="Q52" s="1">
-        <v>52740</v>
+        <v>46240</v>
       </c>
     </row>
     <row r="53" spans="1:17" x14ac:dyDescent="0.35">
@@ -4258,7 +4255,7 @@
         <v>2.41</v>
       </c>
       <c r="Q54" s="1">
-        <v>8845</v>
+        <v>8840</v>
       </c>
     </row>
     <row r="55" spans="1:17" x14ac:dyDescent="0.35">
@@ -4295,7 +4292,7 @@
         <v>25</v>
       </c>
       <c r="M55" s="2" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="N55" s="2" t="s">
         <v>327</v>
@@ -4307,7 +4304,7 @@
         <v>7.18</v>
       </c>
       <c r="Q55" s="1">
-        <v>6506</v>
+        <v>3741</v>
       </c>
     </row>
     <row r="56" spans="1:17" x14ac:dyDescent="0.35">
@@ -4356,7 +4353,7 @@
         <v>20.7</v>
       </c>
       <c r="Q56" s="1">
-        <v>2954</v>
+        <v>3848</v>
       </c>
     </row>
     <row r="57" spans="1:17" x14ac:dyDescent="0.35">
@@ -4405,7 +4402,7 @@
         <v>0.53</v>
       </c>
       <c r="Q57" s="1">
-        <v>8299</v>
+        <v>8234</v>
       </c>
     </row>
     <row r="58" spans="1:17" x14ac:dyDescent="0.35">
@@ -4454,7 +4451,7 @@
         <v>5.32</v>
       </c>
       <c r="Q58" s="1">
-        <v>44356</v>
+        <v>40986</v>
       </c>
     </row>
     <row r="59" spans="1:17" x14ac:dyDescent="0.35">
@@ -4503,7 +4500,7 @@
         <v>12.95</v>
       </c>
       <c r="Q59" s="1">
-        <v>103</v>
+        <v>95</v>
       </c>
     </row>
     <row r="60" spans="1:17" x14ac:dyDescent="0.35">
@@ -4540,14 +4537,20 @@
         <v>64</v>
       </c>
       <c r="M60" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="N60" s="2" t="s">
         <v>357</v>
       </c>
-      <c r="N60" s="2" t="s">
-        <v>358</v>
-      </c>
-      <c r="O60" s="1"/>
-      <c r="P60" s="1"/>
-      <c r="Q60" s="1"/>
+      <c r="O60" s="1">
+        <v>12.5</v>
+      </c>
+      <c r="P60" s="1">
+        <v>12.5</v>
+      </c>
+      <c r="Q60" s="1">
+        <v>66</v>
+      </c>
     </row>
     <row r="61" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A61" s="1"/>
@@ -4555,38 +4558,38 @@
         <v>17</v>
       </c>
       <c r="C61" s="2" t="s">
+        <v>358</v>
+      </c>
+      <c r="D61" s="2" t="s">
         <v>359</v>
       </c>
-      <c r="D61" s="2" t="s">
+      <c r="E61" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F61" s="2" t="s">
         <v>360</v>
-      </c>
-      <c r="E61" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F61" s="2" t="s">
-        <v>361</v>
       </c>
       <c r="G61" s="1"/>
       <c r="H61" s="1">
         <v>1</v>
       </c>
       <c r="I61" s="2" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="J61" s="2" t="s">
         <v>109</v>
       </c>
       <c r="K61" s="2" t="s">
+        <v>362</v>
+      </c>
+      <c r="L61" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M61" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="N61" s="2" t="s">
         <v>363</v>
-      </c>
-      <c r="L61" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M61" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="N61" s="2" t="s">
-        <v>364</v>
       </c>
       <c r="O61" s="1">
         <v>0.52</v>
@@ -4595,7 +4598,7 @@
         <v>0.52</v>
       </c>
       <c r="Q61" s="1">
-        <v>11135</v>
+        <v>11089</v>
       </c>
     </row>
     <row r="62" spans="1:17" x14ac:dyDescent="0.35">
@@ -4604,38 +4607,38 @@
         <v>17</v>
       </c>
       <c r="C62" s="2" t="s">
+        <v>364</v>
+      </c>
+      <c r="D62" s="2" t="s">
         <v>365</v>
       </c>
-      <c r="D62" s="2" t="s">
+      <c r="E62" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F62" s="2" t="s">
         <v>366</v>
-      </c>
-      <c r="E62" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F62" s="2" t="s">
-        <v>367</v>
       </c>
       <c r="G62" s="1"/>
       <c r="H62" s="1">
         <v>1</v>
       </c>
       <c r="I62" s="2" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="J62" s="2" t="s">
         <v>301</v>
       </c>
       <c r="K62" s="2" t="s">
+        <v>368</v>
+      </c>
+      <c r="L62" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M62" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="N62" s="2" t="s">
         <v>369</v>
-      </c>
-      <c r="L62" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M62" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="N62" s="2" t="s">
-        <v>370</v>
       </c>
       <c r="O62" s="1">
         <v>2.42</v>
@@ -4644,7 +4647,7 @@
         <v>2.42</v>
       </c>
       <c r="Q62" s="1">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="63" spans="1:17" x14ac:dyDescent="0.35">
@@ -4653,29 +4656,29 @@
         <v>17</v>
       </c>
       <c r="C63" s="2" t="s">
+        <v>370</v>
+      </c>
+      <c r="D63" s="2" t="s">
         <v>371</v>
       </c>
-      <c r="D63" s="2" t="s">
+      <c r="E63" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F63" s="2" t="s">
         <v>372</v>
-      </c>
-      <c r="E63" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F63" s="2" t="s">
-        <v>373</v>
       </c>
       <c r="G63" s="1"/>
       <c r="H63" s="1">
         <v>1</v>
       </c>
       <c r="I63" s="2" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="J63" s="2" t="s">
         <v>214</v>
       </c>
       <c r="K63" s="2" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="L63" s="2" t="s">
         <v>25</v>
@@ -4684,13 +4687,13 @@
         <v>38</v>
       </c>
       <c r="N63" s="2" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="O63" s="1">
-        <v>2.94</v>
+        <v>2.0699999999999998</v>
       </c>
       <c r="P63" s="1">
-        <v>2.94</v>
+        <v>2.0699999999999998</v>
       </c>
       <c r="Q63" s="1">
         <v>2068</v>
@@ -4702,30 +4705,30 @@
         <v>17</v>
       </c>
       <c r="C64" s="2" t="s">
+        <v>376</v>
+      </c>
+      <c r="D64" s="2" t="s">
         <v>377</v>
       </c>
-      <c r="D64" s="2" t="s">
+      <c r="E64" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F64" s="2" t="s">
         <v>378</v>
-      </c>
-      <c r="E64" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F64" s="2" t="s">
-        <v>379</v>
       </c>
       <c r="G64" s="1"/>
       <c r="H64" s="1">
         <v>1</v>
       </c>
       <c r="I64" s="2" t="s">
+        <v>379</v>
+      </c>
+      <c r="J64" s="2" t="s">
         <v>380</v>
       </c>
-      <c r="J64" s="2" t="s">
+      <c r="K64" s="2" t="s">
         <v>381</v>
       </c>
-      <c r="K64" s="2" t="s">
-        <v>382</v>
-      </c>
       <c r="L64" s="2" t="s">
         <v>25</v>
       </c>
@@ -4733,16 +4736,16 @@
         <v>26</v>
       </c>
       <c r="N64" s="2" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="O64" s="1">
-        <v>0.43</v>
+        <v>0.42</v>
       </c>
       <c r="P64" s="1">
-        <v>0.43</v>
+        <v>0.42</v>
       </c>
       <c r="Q64" s="1">
-        <v>105756</v>
+        <v>219752</v>
       </c>
     </row>
     <row r="65" spans="1:17" x14ac:dyDescent="0.35">
@@ -4751,38 +4754,38 @@
         <v>17</v>
       </c>
       <c r="C65" s="2" t="s">
+        <v>382</v>
+      </c>
+      <c r="D65" s="2" t="s">
         <v>383</v>
       </c>
-      <c r="D65" s="2" t="s">
+      <c r="E65" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F65" s="2" t="s">
         <v>384</v>
-      </c>
-      <c r="E65" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F65" s="2" t="s">
-        <v>385</v>
       </c>
       <c r="G65" s="1"/>
       <c r="H65" s="1">
         <v>1</v>
       </c>
       <c r="I65" s="2" t="s">
+        <v>385</v>
+      </c>
+      <c r="J65" s="2" t="s">
         <v>386</v>
       </c>
-      <c r="J65" s="2" t="s">
+      <c r="K65" s="2" t="s">
         <v>387</v>
       </c>
-      <c r="K65" s="2" t="s">
+      <c r="L65" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M65" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="N65" s="2" t="s">
         <v>388</v>
-      </c>
-      <c r="L65" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M65" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="N65" s="2" t="s">
-        <v>389</v>
       </c>
       <c r="O65" s="1">
         <v>0.56999999999999995</v>
@@ -4791,7 +4794,7 @@
         <v>0.56999999999999995</v>
       </c>
       <c r="Q65" s="1">
-        <v>6070</v>
+        <v>6066</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Generate new fabrication files
</commit_message>
<xml_diff>
--- a/Project Outputs for TSI_SAMP_SAMI_V3.4/Generate Files/BOM/Bill of Materials-TSI_SAMP_SAMI_V3.4(SAMI_V3.5).xlsx
+++ b/Project Outputs for TSI_SAMP_SAMI_V3.4/Generate Files/BOM/Bill of Materials-TSI_SAMP_SAMI_V3.4(SAMI_V3.5).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\biark\Documents\CanAssist\TSI_SAMP_SAMI\Project Outputs for TSI_SAMP_SAMI_V3.4\Generate Files\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Documents\CanAssist\Altium\TSI_SAMP_SAMI\Project Outputs for TSI_SAMP_SAMI_V3.4\Generate Files\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{70EDD994-359F-49BC-9BB6-0B2FFBDCEF49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{87D0E63E-8DF3-4AC8-B8F5-080C03D91BC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2280" yWindow="2280" windowWidth="19200" windowHeight="11170" xr2:uid="{B0082170-DDA8-4935-AA34-F41290B8C798}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{C134B3CD-A938-4DBC-A40F-94F47F66DD4A}"/>
   </bookViews>
   <sheets>
     <sheet name="Bill of Materials-TSI_SAMP_SAMI" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="716" uniqueCount="389">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="715" uniqueCount="386">
   <si>
     <t>Revision ID</t>
   </si>
@@ -155,88 +155,85 @@
     <t>CC0603MRX5R7BB106</t>
   </si>
   <si>
+    <t>311-1822-1-ND</t>
+  </si>
+  <si>
+    <t>1nF</t>
+  </si>
+  <si>
+    <t>CAP CER 0603 1NF 16V X7R 10%</t>
+  </si>
+  <si>
+    <t>C11</t>
+  </si>
+  <si>
+    <t>C0603C102K4RECAUTO</t>
+  </si>
+  <si>
+    <t>399-17878-1-ND</t>
+  </si>
+  <si>
+    <t>1uF</t>
+  </si>
+  <si>
+    <t>0603 1 uF 50 V ±10% Tolerance X5R Surface Mount Multilayer Ceramic Capacitor</t>
+  </si>
+  <si>
+    <t>C13, C14, C20, C24, C27, C29, C30, C31, C57</t>
+  </si>
+  <si>
+    <t>TAIYO YUDEN</t>
+  </si>
+  <si>
+    <t>UMK107BJ105KA-T</t>
+  </si>
+  <si>
+    <t>587-2400-1-ND</t>
+  </si>
+  <si>
+    <t>10µF ±20% 16V Ceramic Capacitor X7R 1206 (3216 Metric)</t>
+  </si>
+  <si>
+    <t>C16, C17</t>
+  </si>
+  <si>
+    <t>CAP-1206</t>
+  </si>
+  <si>
+    <t>Samsung Electro-Mechanics</t>
+  </si>
+  <si>
+    <t>CL31B106MOHNNNE</t>
+  </si>
+  <si>
+    <t>1276-6641-1-ND</t>
+  </si>
+  <si>
+    <t>330uF</t>
+  </si>
+  <si>
+    <t>330µF 50V Aluminum Electrolytic Capacitors Radial, Can - SMD 120mOhm @ 100kHz 5000 Hrs @ 105°C</t>
+  </si>
+  <si>
+    <t>C19, C22</t>
+  </si>
+  <si>
+    <t>CAP ALUM 330UF 20% 50V SMD</t>
+  </si>
+  <si>
+    <t>Wurth Elektronik</t>
+  </si>
+  <si>
+    <t>865080557015</t>
+  </si>
+  <si>
+    <t>Unknown</t>
+  </si>
+  <si>
     <t>Mouser</t>
   </si>
   <si>
-    <t>603-CC603MRX5R7BB106</t>
-  </si>
-  <si>
-    <t>1nF</t>
-  </si>
-  <si>
-    <t>CAP CER 0603 1NF 16V X7R 10%</t>
-  </si>
-  <si>
-    <t>C11</t>
-  </si>
-  <si>
-    <t>KEMET</t>
-  </si>
-  <si>
-    <t>C0603C102K4RECAUTO</t>
-  </si>
-  <si>
-    <t>399-17878-1-ND</t>
-  </si>
-  <si>
-    <t>1uF</t>
-  </si>
-  <si>
-    <t>0603 1 uF 50 V ±10% Tolerance X5R Surface Mount Multilayer Ceramic Capacitor</t>
-  </si>
-  <si>
-    <t>C13, C14, C20, C24, C27, C29, C30, C31, C57</t>
-  </si>
-  <si>
-    <t>TAIYO YUDEN</t>
-  </si>
-  <si>
-    <t>UMK107BJ105KA-T</t>
-  </si>
-  <si>
-    <t>587-2400-1-ND</t>
-  </si>
-  <si>
-    <t>10µF ±20% 16V Ceramic Capacitor X7R 1206 (3216 Metric)</t>
-  </si>
-  <si>
-    <t>C16, C17</t>
-  </si>
-  <si>
-    <t>CAP-1206</t>
-  </si>
-  <si>
-    <t>Samsung Electro-Mechanics</t>
-  </si>
-  <si>
-    <t>CL31B106MOHNNNE</t>
-  </si>
-  <si>
-    <t>1276-6641-1-ND</t>
-  </si>
-  <si>
-    <t>330uF</t>
-  </si>
-  <si>
-    <t>330µF 50V Aluminum Electrolytic Capacitors Radial, Can - SMD 120mOhm @ 100kHz 5000 Hrs @ 105°C</t>
-  </si>
-  <si>
-    <t>C19, C22</t>
-  </si>
-  <si>
-    <t>CAP ALUM 330UF 20% 50V SMD</t>
-  </si>
-  <si>
-    <t>Wurth Elektronik</t>
-  </si>
-  <si>
-    <t>865080557015</t>
-  </si>
-  <si>
-    <t>Unknown</t>
-  </si>
-  <si>
-    <t>732-8514-1-ND</t>
+    <t>710-865080557015</t>
   </si>
   <si>
     <t>2.2uF</t>
@@ -296,7 +293,7 @@
     <t>AC0603JRNPOYBN220</t>
   </si>
   <si>
-    <t>311-3095-1-ND</t>
+    <t>603-AC603JRNPOYBN220</t>
   </si>
   <si>
     <t>15pF</t>
@@ -407,9 +404,6 @@
     <t>LED_0603_SMD</t>
   </si>
   <si>
-    <t>Lite-On</t>
-  </si>
-  <si>
     <t>LTST-C191KGKT</t>
   </si>
   <si>
@@ -488,7 +482,7 @@
     <t>MI0805M221R-10</t>
   </si>
   <si>
-    <t>240-2392-1-ND</t>
+    <t>875-MI0805M221R-10</t>
   </si>
   <si>
     <t>TAG_CONNECT_TC2030</t>
@@ -506,6 +500,24 @@
     <t>TC2030-IDC-ND</t>
   </si>
   <si>
+    <t>16-Pin_B2B</t>
+  </si>
+  <si>
+    <t>Mechanical Part DW-16-07-T-S-200 for use as board to board connector for DS1</t>
+  </si>
+  <si>
+    <t>H2</t>
+  </si>
+  <si>
+    <t>Samtec</t>
+  </si>
+  <si>
+    <t>DW-16-07-T-S-200</t>
+  </si>
+  <si>
+    <t>200-DW1607TS200</t>
+  </si>
+  <si>
     <t>DC_IN</t>
   </si>
   <si>
@@ -581,7 +593,7 @@
     <t>3M</t>
   </si>
   <si>
-    <t>2908-05WB-MG</t>
+    <t>7010506878</t>
   </si>
   <si>
     <t>3M5607CT-ND</t>
@@ -599,7 +611,7 @@
     <t>HDRV5W67P0X254_1X5_1270X241X858P</t>
   </si>
   <si>
-    <t>Amphenol Communications Solutions</t>
+    <t>Amphenol</t>
   </si>
   <si>
     <t>68000-105HTLF</t>
@@ -671,7 +683,7 @@
     <t>DMP2045UQ-7</t>
   </si>
   <si>
-    <t>31-DMP2045UQ-7CT-ND</t>
+    <t>621-DMP2045UQ-7</t>
   </si>
   <si>
     <t>BC848CLT1G</t>
@@ -686,7 +698,7 @@
     <t>onsemi</t>
   </si>
   <si>
-    <t>BC848CLT1GOSDKR-ND</t>
+    <t>863-BC848CLT1G</t>
   </si>
   <si>
     <t>100K</t>
@@ -740,7 +752,7 @@
     <t>RC0603JR-072ML</t>
   </si>
   <si>
-    <t>603-RC0603JR-072ML</t>
+    <t>311-2.0MGRCT-ND</t>
   </si>
   <si>
     <t>20K</t>
@@ -827,10 +839,10 @@
     <t>RES SMD 0 OHM JUMPER 1/10W 0603</t>
   </si>
   <si>
-    <t>R16, R17, R18, R19, R27, R29, R31, R33, R35, R65, R67, R68, R69, R70, R72, R75, R76, R77, R78, R79, R80, R81, R82, R83, R84, R85, R86, R87, R88, R89, R90, R91, R92</t>
-  </si>
-  <si>
-    <t>1623094-1</t>
+    <t>R16, R17, R18, R19, R27, R29, R31, R33, R35, R65, R67, R68, R69, R70, R72</t>
+  </si>
+  <si>
+    <t>CRG0603ZR</t>
   </si>
   <si>
     <t>A106051CT-ND</t>
@@ -971,7 +983,7 @@
     <t>EVQ-Q2U03W</t>
   </si>
   <si>
-    <t>P12955SCT-ND</t>
+    <t>667-EVQ-Q2U03W</t>
   </si>
   <si>
     <t>CONN_TP_SMD</t>
@@ -1022,7 +1034,7 @@
     <t>MAX9744ETH+T</t>
   </si>
   <si>
-    <t>MAX9744ETH+TCT-ND</t>
+    <t>700-MAX9744ETH+T</t>
   </si>
   <si>
     <t>MAX6818EAP+T</t>
@@ -1061,27 +1073,6 @@
     <t>AP7312-1833W6-7DICT-ND</t>
   </si>
   <si>
-    <t>SSR</t>
-  </si>
-  <si>
-    <t>Solid State SPST-NO (1 Form A) 6-SMD, Gull Wing</t>
-  </si>
-  <si>
-    <t>U6, U7, U8, U9</t>
-  </si>
-  <si>
-    <t>IC_SSR_NO_SMD</t>
-  </si>
-  <si>
-    <t>Toshiba</t>
-  </si>
-  <si>
-    <t>TLP170AM(V4TPL,E</t>
-  </si>
-  <si>
-    <t>264-TLP170AM(V4TPLECT-ND</t>
-  </si>
-  <si>
     <t>IC_MDBT50Q-1M_SMD</t>
   </si>
   <si>
@@ -1112,7 +1103,7 @@
     <t>1681</t>
   </si>
   <si>
-    <t>485-1681</t>
+    <t>1528-2645-ND</t>
   </si>
   <si>
     <t>IC BUF ESD</t>
@@ -1601,30 +1592,30 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA7B93E9-26FE-4C90-941D-E8DAC8A59544}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2162314A-A6B2-494A-B28C-0D3AD03DB16C}">
   <dimension ref="A1:Q65"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.81640625" customWidth="1"/>
-    <col min="2" max="2" width="8.81640625" customWidth="1"/>
-    <col min="3" max="3" width="18.81640625" customWidth="1"/>
-    <col min="4" max="4" width="39.453125" customWidth="1"/>
-    <col min="5" max="5" width="15.08984375" customWidth="1"/>
-    <col min="6" max="6" width="25.08984375" customWidth="1"/>
-    <col min="7" max="7" width="16" customWidth="1"/>
-    <col min="8" max="8" width="10.81640625" customWidth="1"/>
-    <col min="9" max="9" width="15.81640625" customWidth="1"/>
-    <col min="10" max="10" width="18.81640625" customWidth="1"/>
-    <col min="11" max="11" width="26.26953125" customWidth="1"/>
-    <col min="12" max="12" width="22.90625" customWidth="1"/>
-    <col min="13" max="13" width="18.81640625" customWidth="1"/>
-    <col min="14" max="14" width="22.1796875" customWidth="1"/>
-    <col min="15" max="15" width="19.90625" customWidth="1"/>
-    <col min="16" max="16" width="19.1796875" customWidth="1"/>
-    <col min="17" max="17" width="19.6328125" customWidth="1"/>
+    <col min="1" max="1" width="19.7109375" customWidth="1"/>
+    <col min="2" max="2" width="9.28515625" customWidth="1"/>
+    <col min="3" max="3" width="19.7109375" customWidth="1"/>
+    <col min="4" max="4" width="41.140625" customWidth="1"/>
+    <col min="5" max="5" width="15.7109375" customWidth="1"/>
+    <col min="6" max="6" width="26.140625" customWidth="1"/>
+    <col min="7" max="7" width="16.7109375" customWidth="1"/>
+    <col min="8" max="8" width="11.28515625" customWidth="1"/>
+    <col min="9" max="9" width="16.5703125" customWidth="1"/>
+    <col min="10" max="10" width="19.7109375" customWidth="1"/>
+    <col min="11" max="11" width="27.42578125" customWidth="1"/>
+    <col min="12" max="12" width="24" customWidth="1"/>
+    <col min="13" max="13" width="19.7109375" customWidth="1"/>
+    <col min="14" max="14" width="23.140625" customWidth="1"/>
+    <col min="15" max="15" width="20.85546875" customWidth="1"/>
+    <col min="16" max="16" width="20" customWidth="1"/>
+    <col min="17" max="17" width="20.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" s="4" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:17" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1677,7 +1668,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
       <c r="B2" s="2" t="s">
         <v>17</v>
@@ -1717,16 +1708,16 @@
         <v>27</v>
       </c>
       <c r="O2" s="1">
-        <v>3.4000000000000002E-2</v>
+        <v>3.5999999999999997E-2</v>
       </c>
       <c r="P2" s="1">
-        <v>0.34</v>
+        <v>0.36</v>
       </c>
       <c r="Q2" s="1">
-        <v>248879</v>
-      </c>
-    </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.35">
+        <v>164272</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="2" t="s">
         <v>17</v>
@@ -1766,16 +1757,16 @@
         <v>33</v>
       </c>
       <c r="O3" s="1">
-        <v>2.5000000000000001E-2</v>
+        <v>2.5999999999999999E-2</v>
       </c>
       <c r="P3" s="1">
-        <v>0.45</v>
+        <v>0.46800000000000003</v>
       </c>
       <c r="Q3" s="1">
-        <v>391</v>
-      </c>
-    </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.35">
+        <v>134606</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
       <c r="B4" s="2" t="s">
         <v>17</v>
@@ -1809,37 +1800,37 @@
         <v>25</v>
       </c>
       <c r="M4" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="N4" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="N4" s="2" t="s">
-        <v>39</v>
-      </c>
       <c r="O4" s="1">
-        <v>0.17499999999999999</v>
+        <v>0.248</v>
       </c>
       <c r="P4" s="1">
-        <v>2.1</v>
+        <v>2.98</v>
       </c>
       <c r="Q4" s="1">
-        <v>17717</v>
-      </c>
-    </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.35">
+        <v>44540</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
       <c r="B5" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C5" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="E5" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F5" s="2" t="s">
         <v>41</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>42</v>
       </c>
       <c r="G5" s="1"/>
       <c r="H5" s="1">
@@ -1849,10 +1840,10 @@
         <v>22</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>43</v>
+        <v>23</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="L5" s="2" t="s">
         <v>25</v>
@@ -1861,7 +1852,7 @@
         <v>26</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="O5" s="1">
         <v>0.13</v>
@@ -1870,25 +1861,25 @@
         <v>0.13</v>
       </c>
       <c r="Q5" s="1">
-        <v>22350</v>
-      </c>
-    </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.35">
+        <v>14988</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
       <c r="B6" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C6" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F6" s="2" t="s">
         <v>46</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>48</v>
       </c>
       <c r="G6" s="1"/>
       <c r="H6" s="1">
@@ -1898,10 +1889,10 @@
         <v>22</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="L6" s="2" t="s">
         <v>25</v>
@@ -1910,19 +1901,19 @@
         <v>26</v>
       </c>
       <c r="N6" s="2" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="O6" s="1">
-        <v>2.3E-2</v>
+        <v>8.6999999999999994E-2</v>
       </c>
       <c r="P6" s="1">
-        <v>0.23</v>
+        <v>0.87</v>
       </c>
       <c r="Q6" s="1">
-        <v>546364</v>
-      </c>
-    </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.35">
+        <v>768633</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
       <c r="B7" s="2" t="s">
         <v>17</v>
@@ -1931,26 +1922,26 @@
         <v>34</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>20</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G7" s="1"/>
       <c r="H7" s="1">
         <v>2</v>
       </c>
       <c r="I7" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="K7" s="2" t="s">
         <v>54</v>
-      </c>
-      <c r="J7" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="K7" s="2" t="s">
-        <v>56</v>
       </c>
       <c r="L7" s="2" t="s">
         <v>25</v>
@@ -1959,83 +1950,83 @@
         <v>26</v>
       </c>
       <c r="N7" s="2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="O7" s="1">
-        <v>0.18</v>
+        <v>0.19</v>
       </c>
       <c r="P7" s="1">
-        <v>0.36</v>
+        <v>0.38</v>
       </c>
       <c r="Q7" s="1">
-        <v>366595</v>
-      </c>
-    </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.35">
+        <v>78849</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8" s="1"/>
       <c r="B8" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C8" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F8" s="2" t="s">
         <v>58</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>60</v>
       </c>
       <c r="G8" s="1"/>
       <c r="H8" s="1">
         <v>2</v>
       </c>
       <c r="I8" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="K8" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="J8" s="2" t="s">
+      <c r="L8" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="K8" s="2" t="s">
+      <c r="M8" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="L8" s="2" t="s">
+      <c r="N8" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="M8" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="N8" s="2" t="s">
-        <v>65</v>
-      </c>
       <c r="O8" s="1">
-        <v>0.97</v>
+        <v>0.98</v>
       </c>
       <c r="P8" s="1">
-        <v>1.94</v>
+        <v>1.96</v>
       </c>
       <c r="Q8" s="1">
-        <v>16225</v>
-      </c>
-    </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.35">
+        <v>2892</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" s="1"/>
       <c r="B9" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C9" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="D9" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="E9" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F9" s="2" t="s">
         <v>67</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>68</v>
       </c>
       <c r="G9" s="1"/>
       <c r="H9" s="1">
@@ -2045,10 +2036,10 @@
         <v>22</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="L9" s="2" t="s">
         <v>25</v>
@@ -2057,83 +2048,83 @@
         <v>26</v>
       </c>
       <c r="N9" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="O9" s="1">
-        <v>0.24</v>
+        <v>0.26</v>
       </c>
       <c r="P9" s="1">
-        <v>0.24</v>
+        <v>0.26</v>
       </c>
       <c r="Q9" s="1">
-        <v>89087</v>
-      </c>
-    </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.35">
+        <v>73982</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A10" s="1"/>
       <c r="B10" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C10" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="D10" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="E10" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F10" s="2" t="s">
         <v>72</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>73</v>
       </c>
       <c r="G10" s="1"/>
       <c r="H10" s="1">
         <v>2</v>
       </c>
       <c r="I10" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="J10" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="K10" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="L10" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M10" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="N10" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="J10" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="K10" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="L10" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M10" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="N10" s="2" t="s">
-        <v>75</v>
-      </c>
       <c r="O10" s="1">
-        <v>0.33</v>
+        <v>0.43</v>
       </c>
       <c r="P10" s="1">
-        <v>0.66</v>
+        <v>0.86</v>
       </c>
       <c r="Q10" s="1">
-        <v>225070</v>
-      </c>
-    </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.35">
+        <v>147988</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" s="1"/>
       <c r="B11" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C11" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D11" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="E11" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F11" s="2" t="s">
         <v>77</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>78</v>
       </c>
       <c r="G11" s="1"/>
       <c r="H11" s="1">
@@ -2143,10 +2134,10 @@
         <v>22</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>43</v>
+        <v>23</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="L11" s="2" t="s">
         <v>25</v>
@@ -2155,34 +2146,34 @@
         <v>26</v>
       </c>
       <c r="N11" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="O11" s="1">
-        <v>0.18</v>
+        <v>0.19</v>
       </c>
       <c r="P11" s="1">
-        <v>0.36</v>
+        <v>0.38</v>
       </c>
       <c r="Q11" s="1">
-        <v>30423</v>
-      </c>
-    </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.35">
+        <v>51083</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" s="1"/>
       <c r="B12" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C12" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="E12" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F12" s="2" t="s">
         <v>82</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>83</v>
       </c>
       <c r="G12" s="1"/>
       <c r="H12" s="1">
@@ -2195,43 +2186,43 @@
         <v>23</v>
       </c>
       <c r="K12" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="L12" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M12" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="N12" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="L12" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M12" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="N12" s="2" t="s">
-        <v>85</v>
-      </c>
       <c r="O12" s="1">
-        <v>0.16</v>
+        <v>0.18</v>
       </c>
       <c r="P12" s="1">
-        <v>0.32</v>
+        <v>0.36</v>
       </c>
       <c r="Q12" s="1">
-        <v>1441</v>
-      </c>
-    </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.35">
+        <v>79342</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" s="1"/>
       <c r="B13" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C13" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F13" s="2" t="s">
         <v>86</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>87</v>
       </c>
       <c r="G13" s="1"/>
       <c r="H13" s="1">
@@ -2244,7 +2235,7 @@
         <v>31</v>
       </c>
       <c r="K13" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="L13" s="2" t="s">
         <v>25</v>
@@ -2253,7 +2244,7 @@
         <v>26</v>
       </c>
       <c r="N13" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="O13" s="1">
         <v>0.1</v>
@@ -2262,25 +2253,25 @@
         <v>0.2</v>
       </c>
       <c r="Q13" s="1">
-        <v>28107</v>
-      </c>
-    </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.35">
+        <v>23983</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A14" s="1"/>
       <c r="B14" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C14" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="D14" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="E14" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F14" s="2" t="s">
         <v>91</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>92</v>
       </c>
       <c r="G14" s="1"/>
       <c r="H14" s="1">
@@ -2290,10 +2281,10 @@
         <v>22</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>43</v>
+        <v>23</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="L14" s="2" t="s">
         <v>25</v>
@@ -2302,34 +2293,34 @@
         <v>26</v>
       </c>
       <c r="N14" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="O14" s="1">
-        <v>0.35</v>
+        <v>0.37</v>
       </c>
       <c r="P14" s="1">
-        <v>0.7</v>
+        <v>0.74</v>
       </c>
       <c r="Q14" s="1">
-        <v>52423</v>
-      </c>
-    </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.35">
+        <v>141787</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15" s="1"/>
       <c r="B15" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C15" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="D15" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="D15" s="2" t="s">
+      <c r="E15" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F15" s="2" t="s">
         <v>96</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>97</v>
       </c>
       <c r="G15" s="1"/>
       <c r="H15" s="1">
@@ -2339,10 +2330,10 @@
         <v>22</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>43</v>
+        <v>23</v>
       </c>
       <c r="K15" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="L15" s="2" t="s">
         <v>25</v>
@@ -2351,7 +2342,7 @@
         <v>26</v>
       </c>
       <c r="N15" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="O15" s="1">
         <v>0.1</v>
@@ -2360,25 +2351,25 @@
         <v>0.1</v>
       </c>
       <c r="Q15" s="1">
-        <v>678834</v>
-      </c>
-    </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.35">
+        <v>532488</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A16" s="1"/>
       <c r="B16" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C16" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D16" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="D16" s="2" t="s">
+      <c r="E16" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F16" s="2" t="s">
         <v>101</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>102</v>
       </c>
       <c r="G16" s="1"/>
       <c r="H16" s="1">
@@ -2388,59 +2379,59 @@
         <v>22</v>
       </c>
       <c r="J16" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="K16" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="L16" s="2" t="s">
         <v>62</v>
-      </c>
-      <c r="K16" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="L16" s="2" t="s">
-        <v>64</v>
       </c>
       <c r="M16" s="2" t="s">
         <v>26</v>
       </c>
       <c r="N16" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="O16" s="1">
-        <v>0.1</v>
+        <v>0.11</v>
       </c>
       <c r="P16" s="1">
-        <v>0.2</v>
+        <v>0.22</v>
       </c>
       <c r="Q16" s="1">
-        <v>13365</v>
-      </c>
-    </row>
-    <row r="17" spans="1:17" x14ac:dyDescent="0.35">
+        <v>11303</v>
+      </c>
+    </row>
+    <row r="17" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A17" s="1"/>
       <c r="B17" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C17" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D17" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="D17" s="2" t="s">
+      <c r="E17" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F17" s="2" t="s">
         <v>106</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>107</v>
       </c>
       <c r="G17" s="1"/>
       <c r="H17" s="1">
         <v>2</v>
       </c>
       <c r="I17" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="J17" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="J17" s="2" t="s">
-        <v>109</v>
-      </c>
       <c r="K17" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="L17" s="2" t="s">
         <v>25</v>
@@ -2449,47 +2440,47 @@
         <v>26</v>
       </c>
       <c r="N17" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="O17" s="1">
-        <v>1.58</v>
+        <v>1.67</v>
       </c>
       <c r="P17" s="1">
-        <v>3.16</v>
+        <v>3.34</v>
       </c>
       <c r="Q17" s="1">
-        <v>20394</v>
-      </c>
-    </row>
-    <row r="18" spans="1:17" x14ac:dyDescent="0.35">
+        <v>52293</v>
+      </c>
+    </row>
+    <row r="18" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" s="1"/>
       <c r="B18" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C18" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="D18" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="D18" s="2" t="s">
+      <c r="E18" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F18" s="2" t="s">
         <v>112</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F18" s="2" t="s">
-        <v>113</v>
       </c>
       <c r="G18" s="1"/>
       <c r="H18" s="1">
         <v>1</v>
       </c>
       <c r="I18" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="J18" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="J18" s="2" t="s">
+      <c r="K18" s="2" t="s">
         <v>115</v>
-      </c>
-      <c r="K18" s="2" t="s">
-        <v>116</v>
       </c>
       <c r="L18" s="2" t="s">
         <v>25</v>
@@ -2498,47 +2489,47 @@
         <v>26</v>
       </c>
       <c r="N18" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="O18" s="1">
-        <v>0.39</v>
+        <v>0.74</v>
       </c>
       <c r="P18" s="1">
-        <v>0.39</v>
+        <v>0.74</v>
       </c>
       <c r="Q18" s="1">
-        <v>28281</v>
-      </c>
-    </row>
-    <row r="19" spans="1:17" x14ac:dyDescent="0.35">
+        <v>35275</v>
+      </c>
+    </row>
+    <row r="19" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A19" s="1"/>
       <c r="B19" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C19" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="D19" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="D19" s="2" t="s">
+      <c r="E19" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F19" s="2" t="s">
         <v>119</v>
-      </c>
-      <c r="E19" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F19" s="2" t="s">
-        <v>120</v>
       </c>
       <c r="G19" s="1"/>
       <c r="H19" s="1">
         <v>1</v>
       </c>
       <c r="I19" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="J19" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="K19" s="2" t="s">
         <v>121</v>
-      </c>
-      <c r="J19" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="K19" s="2" t="s">
-        <v>123</v>
       </c>
       <c r="L19" s="2" t="s">
         <v>25</v>
@@ -2547,7 +2538,7 @@
         <v>26</v>
       </c>
       <c r="N19" s="2" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="O19" s="1">
         <v>0.15</v>
@@ -2556,38 +2547,38 @@
         <v>0.15</v>
       </c>
       <c r="Q19" s="1">
-        <v>1321305</v>
-      </c>
-    </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.35">
+        <v>1126158</v>
+      </c>
+    </row>
+    <row r="20" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A20" s="1"/>
       <c r="B20" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C20" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F20" s="2" t="s">
         <v>125</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="E20" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F20" s="2" t="s">
-        <v>127</v>
       </c>
       <c r="G20" s="1"/>
       <c r="H20" s="1">
         <v>2</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="J20" s="2" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="K20" s="2" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="L20" s="2" t="s">
         <v>25</v>
@@ -2596,56 +2587,56 @@
         <v>26</v>
       </c>
       <c r="N20" s="2" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="O20" s="1">
-        <v>0.15</v>
+        <v>0.13</v>
       </c>
       <c r="P20" s="1">
-        <v>0.3</v>
+        <v>0.26</v>
       </c>
       <c r="Q20" s="1">
-        <v>386999</v>
-      </c>
-    </row>
-    <row r="21" spans="1:17" x14ac:dyDescent="0.35">
+        <v>776778</v>
+      </c>
+    </row>
+    <row r="21" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A21" s="1"/>
       <c r="B21" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C21" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F21" s="2" t="s">
         <v>130</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="E21" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F21" s="2" t="s">
-        <v>132</v>
       </c>
       <c r="G21" s="1"/>
       <c r="H21" s="1">
         <v>1</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="J21" s="2" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="K21" s="2" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="L21" s="2" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="M21" s="2" t="s">
         <v>26</v>
       </c>
       <c r="N21" s="2" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="O21" s="1">
         <v>35.450000000000003</v>
@@ -2654,38 +2645,38 @@
         <v>35.450000000000003</v>
       </c>
       <c r="Q21" s="1">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="22" spans="1:17" x14ac:dyDescent="0.35">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="22" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A22" s="1"/>
       <c r="B22" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C22" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F22" s="2" t="s">
         <v>136</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="E22" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F22" s="2" t="s">
-        <v>138</v>
       </c>
       <c r="G22" s="1"/>
       <c r="H22" s="1">
         <v>3</v>
       </c>
       <c r="I22" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="J22" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="K22" s="2" t="s">
         <v>139</v>
-      </c>
-      <c r="J22" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="K22" s="2" t="s">
-        <v>141</v>
       </c>
       <c r="L22" s="2" t="s">
         <v>25</v>
@@ -2694,56 +2685,56 @@
         <v>26</v>
       </c>
       <c r="N22" s="2" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="O22" s="1">
-        <v>0.28999999999999998</v>
+        <v>0.31</v>
       </c>
       <c r="P22" s="1">
-        <v>0.87</v>
+        <v>0.93</v>
       </c>
       <c r="Q22" s="1">
-        <v>53673</v>
-      </c>
-    </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.35">
+        <v>1766</v>
+      </c>
+    </row>
+    <row r="23" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A23" s="1"/>
       <c r="B23" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C23" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F23" s="2" t="s">
         <v>143</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="E23" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F23" s="2" t="s">
-        <v>145</v>
       </c>
       <c r="G23" s="1"/>
       <c r="H23" s="1">
         <v>4</v>
       </c>
       <c r="I23" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="J23" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="K23" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="J23" s="2" t="s">
+      <c r="L23" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M23" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="N23" s="2" t="s">
         <v>147</v>
-      </c>
-      <c r="K23" s="2" t="s">
-        <v>148</v>
-      </c>
-      <c r="L23" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M23" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="N23" s="2" t="s">
-        <v>149</v>
       </c>
       <c r="O23" s="1">
         <v>0.1</v>
@@ -2752,234 +2743,232 @@
         <v>0.4</v>
       </c>
       <c r="Q23" s="1">
-        <v>50115</v>
-      </c>
-    </row>
-    <row r="24" spans="1:17" x14ac:dyDescent="0.35">
+        <v>48646</v>
+      </c>
+    </row>
+    <row r="24" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A24" s="1"/>
       <c r="B24" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C24" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F24" s="2" t="s">
         <v>150</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>151</v>
-      </c>
-      <c r="E24" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F24" s="2" t="s">
-        <v>152</v>
       </c>
       <c r="G24" s="1"/>
       <c r="H24" s="1">
         <v>1</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="J24" s="2" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="K24" s="2" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="L24" s="2" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="M24" s="2" t="s">
         <v>26</v>
       </c>
       <c r="N24" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="O24" s="1">
+        <v>44.58</v>
+      </c>
+      <c r="P24" s="1">
+        <v>44.58</v>
+      </c>
+      <c r="Q24" s="1">
+        <v>1926</v>
+      </c>
+    </row>
+    <row r="25" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A25" s="1"/>
+      <c r="B25" s="1"/>
+      <c r="C25" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="D25" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="O24" s="1">
-        <v>43.71</v>
-      </c>
-      <c r="P24" s="1">
-        <v>43.71</v>
-      </c>
-      <c r="Q24" s="1">
-        <v>2009</v>
-      </c>
-    </row>
-    <row r="25" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="A25" s="1"/>
-      <c r="B25" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C25" s="2" t="s">
+      <c r="E25" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F25" s="2" t="s">
         <v>155</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>156</v>
-      </c>
-      <c r="E25" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F25" s="2" t="s">
-        <v>157</v>
       </c>
       <c r="G25" s="1"/>
       <c r="H25" s="1">
         <v>1</v>
       </c>
       <c r="I25" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J25" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="K25" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="L25" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M25" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="N25" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="J25" s="2" t="s">
-        <v>159</v>
-      </c>
-      <c r="K25" s="2" t="s">
-        <v>160</v>
-      </c>
-      <c r="L25" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M25" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="N25" s="2" t="s">
-        <v>161</v>
-      </c>
       <c r="O25" s="1">
-        <v>0.83</v>
+        <v>1.03</v>
       </c>
       <c r="P25" s="1">
-        <v>0.83</v>
+        <v>1.03</v>
       </c>
       <c r="Q25" s="1">
-        <v>8212</v>
-      </c>
-    </row>
-    <row r="26" spans="1:17" x14ac:dyDescent="0.35">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="26" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A26" s="1"/>
       <c r="B26" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>20</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="G26" s="1"/>
       <c r="H26" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I26" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="J26" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="K26" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="L26" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M26" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="N26" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="J26" s="2" t="s">
-        <v>159</v>
-      </c>
-      <c r="K26" s="2" t="s">
-        <v>166</v>
-      </c>
-      <c r="L26" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M26" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="N26" s="2" t="s">
-        <v>167</v>
-      </c>
       <c r="O26" s="1">
-        <v>1.69</v>
+        <v>0.9</v>
       </c>
       <c r="P26" s="1">
-        <v>5.07</v>
+        <v>0.9</v>
       </c>
       <c r="Q26" s="1">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="27" spans="1:17" x14ac:dyDescent="0.35">
+        <v>9534</v>
+      </c>
+    </row>
+    <row r="27" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A27" s="1"/>
       <c r="B27" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C27" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F27" s="2" t="s">
         <v>168</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="E27" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F27" s="2" t="s">
-        <v>169</v>
       </c>
       <c r="G27" s="1"/>
       <c r="H27" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I27" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="J27" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="K27" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="J27" s="2" t="s">
+      <c r="L27" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M27" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="N27" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="K27" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="L27" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M27" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="N27" s="2" t="s">
-        <v>173</v>
-      </c>
       <c r="O27" s="1">
-        <v>1.81</v>
+        <v>1.88</v>
       </c>
       <c r="P27" s="1">
-        <v>3.62</v>
+        <v>5.64</v>
       </c>
       <c r="Q27" s="1">
-        <v>29500</v>
-      </c>
-    </row>
-    <row r="28" spans="1:17" x14ac:dyDescent="0.35">
+        <v>2589</v>
+      </c>
+    </row>
+    <row r="28" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A28" s="1"/>
       <c r="B28" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>20</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G28" s="1"/>
       <c r="H28" s="1">
         <v>2</v>
       </c>
       <c r="I28" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="J28" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="J28" s="2" t="s">
-        <v>171</v>
-      </c>
       <c r="K28" s="2" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="L28" s="2" t="s">
         <v>25</v>
@@ -2988,28 +2977,28 @@
         <v>26</v>
       </c>
       <c r="N28" s="2" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="O28" s="1">
-        <v>1.81</v>
+        <v>2.17</v>
       </c>
       <c r="P28" s="1">
-        <v>3.62</v>
+        <v>4.34</v>
       </c>
       <c r="Q28" s="1">
-        <v>29500</v>
-      </c>
-    </row>
-    <row r="29" spans="1:17" x14ac:dyDescent="0.35">
+        <v>22279</v>
+      </c>
+    </row>
+    <row r="29" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A29" s="1"/>
       <c r="B29" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>177</v>
+        <v>167</v>
       </c>
       <c r="E29" s="2" t="s">
         <v>20</v>
@@ -3019,150 +3008,150 @@
       </c>
       <c r="G29" s="1"/>
       <c r="H29" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I29" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="J29" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="K29" s="2" t="s">
         <v>176</v>
       </c>
-      <c r="J29" s="2" t="s">
-        <v>179</v>
-      </c>
-      <c r="K29" s="2" t="s">
-        <v>180</v>
-      </c>
       <c r="L29" s="2" t="s">
-        <v>64</v>
+        <v>25</v>
       </c>
       <c r="M29" s="2" t="s">
         <v>26</v>
       </c>
       <c r="N29" s="2" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="O29" s="1">
-        <v>4.43</v>
+        <v>2.17</v>
       </c>
       <c r="P29" s="1">
-        <v>4.43</v>
+        <v>4.34</v>
       </c>
       <c r="Q29" s="1">
-        <v>36612</v>
-      </c>
-    </row>
-    <row r="30" spans="1:17" x14ac:dyDescent="0.35">
+        <v>22279</v>
+      </c>
+    </row>
+    <row r="30" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A30" s="1"/>
       <c r="B30" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C30" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F30" s="2" t="s">
         <v>182</v>
-      </c>
-      <c r="D30" s="2" t="s">
-        <v>183</v>
-      </c>
-      <c r="E30" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F30" s="2" t="s">
-        <v>184</v>
       </c>
       <c r="G30" s="1"/>
       <c r="H30" s="1">
         <v>1</v>
       </c>
       <c r="I30" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="J30" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="K30" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="L30" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="M30" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="N30" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="J30" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="K30" s="2" t="s">
-        <v>187</v>
-      </c>
-      <c r="L30" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M30" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="N30" s="2" t="s">
-        <v>188</v>
-      </c>
       <c r="O30" s="1">
-        <v>0.51</v>
+        <v>4.43</v>
       </c>
       <c r="P30" s="1">
-        <v>0.51</v>
+        <v>4.43</v>
       </c>
       <c r="Q30" s="1">
-        <v>3760</v>
-      </c>
-    </row>
-    <row r="31" spans="1:17" x14ac:dyDescent="0.35">
+        <v>26091</v>
+      </c>
+    </row>
+    <row r="31" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A31" s="1"/>
       <c r="B31" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="E31" s="2" t="s">
         <v>20</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="G31" s="1"/>
       <c r="H31" s="1">
         <v>1</v>
       </c>
       <c r="I31" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="J31" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="K31" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="L31" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M31" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="N31" s="2" t="s">
         <v>192</v>
       </c>
-      <c r="J31" s="2" t="s">
-        <v>193</v>
-      </c>
-      <c r="K31" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="L31" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="M31" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="N31" s="2" t="s">
-        <v>195</v>
-      </c>
       <c r="O31" s="1">
-        <v>0.81</v>
+        <v>0.6</v>
       </c>
       <c r="P31" s="1">
-        <v>0.81</v>
+        <v>0.6</v>
       </c>
       <c r="Q31" s="1">
-        <v>216932</v>
-      </c>
-    </row>
-    <row r="32" spans="1:17" x14ac:dyDescent="0.35">
+        <v>3750</v>
+      </c>
+    </row>
+    <row r="32" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A32" s="1"/>
       <c r="B32" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="E32" s="2" t="s">
         <v>20</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="G32" s="1"/>
       <c r="H32" s="1">
@@ -3172,80 +3161,80 @@
         <v>196</v>
       </c>
       <c r="J32" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="K32" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="L32" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="M32" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="N32" s="2" t="s">
         <v>199</v>
       </c>
-      <c r="K32" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="L32" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M32" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="N32" s="2" t="s">
-        <v>200</v>
-      </c>
       <c r="O32" s="1">
-        <v>2.78</v>
+        <v>0.75</v>
       </c>
       <c r="P32" s="1">
-        <v>2.78</v>
+        <v>0.75</v>
       </c>
       <c r="Q32" s="1">
-        <v>4822</v>
-      </c>
-    </row>
-    <row r="33" spans="1:17" x14ac:dyDescent="0.35">
+        <v>124884</v>
+      </c>
+    </row>
+    <row r="33" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A33" s="1"/>
       <c r="B33" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C33" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="D33" s="2" t="s">
         <v>201</v>
       </c>
-      <c r="D33" s="2" t="s">
+      <c r="E33" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F33" s="2" t="s">
         <v>202</v>
-      </c>
-      <c r="E33" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F33" s="2" t="s">
-        <v>203</v>
       </c>
       <c r="G33" s="1"/>
       <c r="H33" s="1">
         <v>1</v>
       </c>
       <c r="I33" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="J33" s="2" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="K33" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="L33" s="2" t="s">
         <v>25</v>
       </c>
       <c r="M33" s="2" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="N33" s="2" t="s">
         <v>204</v>
       </c>
       <c r="O33" s="1">
-        <v>1.4</v>
+        <v>2.86</v>
       </c>
       <c r="P33" s="1">
-        <v>1.4</v>
+        <v>2.86</v>
       </c>
       <c r="Q33" s="1">
-        <v>15307</v>
-      </c>
-    </row>
-    <row r="34" spans="1:17" x14ac:dyDescent="0.35">
+        <v>3483</v>
+      </c>
+    </row>
+    <row r="34" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A34" s="1"/>
       <c r="B34" s="2" t="s">
         <v>17</v>
@@ -3267,160 +3256,160 @@
         <v>1</v>
       </c>
       <c r="I34" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="J34" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="K34" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="L34" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M34" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="N34" s="2" t="s">
         <v>208</v>
       </c>
-      <c r="J34" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="K34" s="2" t="s">
-        <v>209</v>
-      </c>
-      <c r="L34" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M34" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="N34" s="2" t="s">
-        <v>210</v>
-      </c>
       <c r="O34" s="1">
-        <v>0.49</v>
+        <v>1.44</v>
       </c>
       <c r="P34" s="1">
-        <v>0.49</v>
+        <v>1.44</v>
       </c>
       <c r="Q34" s="1">
-        <v>4000</v>
-      </c>
-    </row>
-    <row r="35" spans="1:17" x14ac:dyDescent="0.35">
+        <v>7044</v>
+      </c>
+    </row>
+    <row r="35" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A35" s="1"/>
       <c r="B35" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C35" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="E35" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F35" s="2" t="s">
         <v>211</v>
-      </c>
-      <c r="D35" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E35" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F35" s="2" t="s">
-        <v>212</v>
       </c>
       <c r="G35" s="1"/>
       <c r="H35" s="1">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I35" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="J35" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="K35" s="2" t="s">
         <v>213</v>
       </c>
-      <c r="J35" s="2" t="s">
+      <c r="L35" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M35" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="N35" s="2" t="s">
         <v>214</v>
       </c>
-      <c r="K35" s="2" t="s">
-        <v>211</v>
-      </c>
-      <c r="L35" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M35" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="N35" s="2" t="s">
-        <v>215</v>
-      </c>
       <c r="O35" s="1">
-        <v>0.12</v>
+        <v>0.49</v>
       </c>
       <c r="P35" s="1">
-        <v>0.48</v>
+        <v>0.49</v>
       </c>
       <c r="Q35" s="1">
-        <v>104482</v>
-      </c>
-    </row>
-    <row r="36" spans="1:17" x14ac:dyDescent="0.35">
+        <v>21569</v>
+      </c>
+    </row>
+    <row r="36" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A36" s="1"/>
       <c r="B36" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C36" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F36" s="2" t="s">
         <v>216</v>
-      </c>
-      <c r="D36" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="E36" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F36" s="2" t="s">
-        <v>218</v>
       </c>
       <c r="G36" s="1"/>
       <c r="H36" s="1">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="I36" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="J36" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="K36" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="L36" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M36" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="N36" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="J36" s="2" t="s">
-        <v>220</v>
-      </c>
-      <c r="K36" s="2" t="s">
-        <v>221</v>
-      </c>
-      <c r="L36" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M36" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="N36" s="2" t="s">
-        <v>222</v>
-      </c>
       <c r="O36" s="1">
-        <v>6.9000000000000006E-2</v>
+        <v>0.13</v>
       </c>
       <c r="P36" s="1">
-        <v>0.69</v>
+        <v>0.52</v>
       </c>
       <c r="Q36" s="1">
-        <v>105743</v>
-      </c>
-    </row>
-    <row r="37" spans="1:17" x14ac:dyDescent="0.35">
+        <v>62472</v>
+      </c>
+    </row>
+    <row r="37" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A37" s="1"/>
       <c r="B37" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="E37" s="2" t="s">
         <v>20</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="G37" s="1"/>
       <c r="H37" s="1">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="I37" s="2" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="J37" s="2" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="K37" s="2" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="L37" s="2" t="s">
         <v>25</v>
@@ -3429,56 +3418,56 @@
         <v>26</v>
       </c>
       <c r="N37" s="2" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="O37" s="1">
-        <v>0.1</v>
+        <v>7.2999999999999995E-2</v>
       </c>
       <c r="P37" s="1">
-        <v>0.1</v>
+        <v>0.73</v>
       </c>
       <c r="Q37" s="1">
-        <v>12828</v>
-      </c>
-    </row>
-    <row r="38" spans="1:17" x14ac:dyDescent="0.35">
+        <v>103939</v>
+      </c>
+    </row>
+    <row r="38" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A38" s="1"/>
       <c r="B38" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C38" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F38" s="2" t="s">
         <v>229</v>
-      </c>
-      <c r="D38" s="2" t="s">
-        <v>230</v>
-      </c>
-      <c r="E38" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F38" s="2" t="s">
-        <v>231</v>
       </c>
       <c r="G38" s="1"/>
       <c r="H38" s="1">
         <v>1</v>
       </c>
       <c r="I38" s="2" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="J38" s="2" t="s">
-        <v>23</v>
+        <v>230</v>
       </c>
       <c r="K38" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="L38" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M38" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="N38" s="2" t="s">
         <v>232</v>
-      </c>
-      <c r="L38" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M38" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="N38" s="2" t="s">
-        <v>233</v>
       </c>
       <c r="O38" s="1">
         <v>0.1</v>
@@ -3487,38 +3476,38 @@
         <v>0.1</v>
       </c>
       <c r="Q38" s="1">
-        <v>40267</v>
-      </c>
-    </row>
-    <row r="39" spans="1:17" x14ac:dyDescent="0.35">
+        <v>12818</v>
+      </c>
+    </row>
+    <row r="39" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A39" s="1"/>
       <c r="B39" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C39" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="D39" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="D39" s="2" t="s">
+      <c r="E39" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F39" s="2" t="s">
         <v>235</v>
-      </c>
-      <c r="E39" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F39" s="2" t="s">
-        <v>236</v>
       </c>
       <c r="G39" s="1"/>
       <c r="H39" s="1">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I39" s="2" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="J39" s="2" t="s">
-        <v>226</v>
+        <v>23</v>
       </c>
       <c r="K39" s="2" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="L39" s="2" t="s">
         <v>25</v>
@@ -3527,145 +3516,145 @@
         <v>26</v>
       </c>
       <c r="N39" s="2" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="O39" s="1">
-        <v>7.0000000000000001E-3</v>
+        <v>0.1</v>
       </c>
       <c r="P39" s="1">
-        <v>7.0000000000000007E-2</v>
+        <v>0.1</v>
       </c>
       <c r="Q39" s="1">
-        <v>2710093</v>
-      </c>
-    </row>
-    <row r="40" spans="1:17" x14ac:dyDescent="0.35">
+        <v>108031</v>
+      </c>
+    </row>
+    <row r="40" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A40" s="1"/>
       <c r="B40" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C40" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="D40" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="D40" s="2" t="s">
+      <c r="E40" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F40" s="2" t="s">
         <v>240</v>
-      </c>
-      <c r="E40" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F40" s="2" t="s">
-        <v>241</v>
       </c>
       <c r="G40" s="1"/>
       <c r="H40" s="1">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I40" s="2" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="J40" s="2" t="s">
-        <v>23</v>
+        <v>230</v>
       </c>
       <c r="K40" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="L40" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M40" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="N40" s="2" t="s">
         <v>242</v>
       </c>
-      <c r="L40" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M40" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="N40" s="2" t="s">
-        <v>243</v>
-      </c>
       <c r="O40" s="1">
-        <v>0.1</v>
+        <v>2.1000000000000001E-2</v>
       </c>
       <c r="P40" s="1">
-        <v>0.1</v>
+        <v>0.21</v>
       </c>
       <c r="Q40" s="1">
-        <v>58506</v>
-      </c>
-    </row>
-    <row r="41" spans="1:17" x14ac:dyDescent="0.35">
+        <v>2363400</v>
+      </c>
+    </row>
+    <row r="41" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A41" s="1"/>
       <c r="B41" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C41" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="D41" s="2" t="s">
         <v>244</v>
       </c>
-      <c r="D41" s="2" t="s">
+      <c r="E41" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F41" s="2" t="s">
         <v>245</v>
-      </c>
-      <c r="E41" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F41" s="2" t="s">
-        <v>246</v>
       </c>
       <c r="G41" s="1"/>
       <c r="H41" s="1">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="I41" s="2" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="J41" s="2" t="s">
-        <v>226</v>
+        <v>23</v>
       </c>
       <c r="K41" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="L41" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M41" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="N41" s="2" t="s">
         <v>247</v>
       </c>
-      <c r="L41" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M41" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="N41" s="2" t="s">
-        <v>248</v>
-      </c>
       <c r="O41" s="1">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="P41" s="1">
-        <v>0.18</v>
+        <v>0.1</v>
       </c>
       <c r="Q41" s="1">
-        <v>6562551</v>
-      </c>
-    </row>
-    <row r="42" spans="1:17" x14ac:dyDescent="0.35">
+        <v>39759</v>
+      </c>
+    </row>
+    <row r="42" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A42" s="1"/>
       <c r="B42" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C42" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="D42" s="2" t="s">
         <v>249</v>
       </c>
-      <c r="D42" s="2" t="s">
+      <c r="E42" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F42" s="2" t="s">
         <v>250</v>
-      </c>
-      <c r="E42" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F42" s="2" t="s">
-        <v>251</v>
       </c>
       <c r="G42" s="1"/>
       <c r="H42" s="1">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="I42" s="2" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="J42" s="2" t="s">
-        <v>252</v>
+        <v>230</v>
       </c>
       <c r="K42" s="2" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="L42" s="2" t="s">
         <v>25</v>
@@ -3674,47 +3663,47 @@
         <v>26</v>
       </c>
       <c r="N42" s="2" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="O42" s="1">
-        <v>0.1</v>
+        <v>2.1000000000000001E-2</v>
       </c>
       <c r="P42" s="1">
-        <v>0.2</v>
+        <v>0.378</v>
       </c>
       <c r="Q42" s="1">
-        <v>62060</v>
-      </c>
-    </row>
-    <row r="43" spans="1:17" x14ac:dyDescent="0.35">
+        <v>2483403</v>
+      </c>
+    </row>
+    <row r="43" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A43" s="1"/>
       <c r="B43" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C43" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="E43" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F43" s="2" t="s">
         <v>255</v>
-      </c>
-      <c r="D43" s="2" t="s">
-        <v>256</v>
-      </c>
-      <c r="E43" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F43" s="2" t="s">
-        <v>257</v>
       </c>
       <c r="G43" s="1"/>
       <c r="H43" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I43" s="2" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="J43" s="2" t="s">
-        <v>220</v>
+        <v>256</v>
       </c>
       <c r="K43" s="2" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="L43" s="2" t="s">
         <v>25</v>
@@ -3723,47 +3712,47 @@
         <v>26</v>
       </c>
       <c r="N43" s="2" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="O43" s="1">
-        <v>2.9000000000000001E-2</v>
+        <v>0.1</v>
       </c>
       <c r="P43" s="1">
-        <v>0.28999999999999998</v>
+        <v>0.2</v>
       </c>
       <c r="Q43" s="1">
-        <v>571540</v>
-      </c>
-    </row>
-    <row r="44" spans="1:17" x14ac:dyDescent="0.35">
+        <v>180479</v>
+      </c>
+    </row>
+    <row r="44" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A44" s="1"/>
       <c r="B44" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C44" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="D44" s="2" t="s">
         <v>260</v>
       </c>
-      <c r="D44" s="2" t="s">
+      <c r="E44" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F44" s="2" t="s">
         <v>261</v>
-      </c>
-      <c r="E44" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F44" s="2" t="s">
-        <v>262</v>
       </c>
       <c r="G44" s="1"/>
       <c r="H44" s="1">
-        <v>33</v>
+        <v>3</v>
       </c>
       <c r="I44" s="2" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="J44" s="2" t="s">
-        <v>252</v>
+        <v>224</v>
       </c>
       <c r="K44" s="2" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="L44" s="2" t="s">
         <v>25</v>
@@ -3772,47 +3761,47 @@
         <v>26</v>
       </c>
       <c r="N44" s="2" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="O44" s="1">
-        <v>9.5999999999999992E-3</v>
+        <v>0.1</v>
       </c>
       <c r="P44" s="1">
-        <v>0.31680000000000003</v>
+        <v>0.3</v>
       </c>
       <c r="Q44" s="1">
-        <v>80639</v>
-      </c>
-    </row>
-    <row r="45" spans="1:17" x14ac:dyDescent="0.35">
+        <v>374812</v>
+      </c>
+    </row>
+    <row r="45" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A45" s="1"/>
       <c r="B45" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C45" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="D45" s="2" t="s">
         <v>265</v>
       </c>
-      <c r="D45" s="2" t="s">
+      <c r="E45" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F45" s="2" t="s">
         <v>266</v>
-      </c>
-      <c r="E45" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F45" s="2" t="s">
-        <v>267</v>
       </c>
       <c r="G45" s="1"/>
       <c r="H45" s="1">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="I45" s="2" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="J45" s="2" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="K45" s="2" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="L45" s="2" t="s">
         <v>25</v>
@@ -3821,47 +3810,47 @@
         <v>26</v>
       </c>
       <c r="N45" s="2" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="O45" s="1">
-        <v>0.17</v>
+        <v>1.0999999999999999E-2</v>
       </c>
       <c r="P45" s="1">
-        <v>0.34</v>
+        <v>0.16500000000000001</v>
       </c>
       <c r="Q45" s="1">
-        <v>125657</v>
-      </c>
-    </row>
-    <row r="46" spans="1:17" x14ac:dyDescent="0.35">
+        <v>104304</v>
+      </c>
+    </row>
+    <row r="46" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A46" s="1"/>
       <c r="B46" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C46" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="D46" s="2" t="s">
         <v>270</v>
       </c>
-      <c r="D46" s="2" t="s">
+      <c r="E46" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F46" s="2" t="s">
         <v>271</v>
-      </c>
-      <c r="E46" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F46" s="2" t="s">
-        <v>272</v>
       </c>
       <c r="G46" s="1"/>
       <c r="H46" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I46" s="2" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="J46" s="2" t="s">
-        <v>23</v>
+        <v>256</v>
       </c>
       <c r="K46" s="2" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="L46" s="2" t="s">
         <v>25</v>
@@ -3870,47 +3859,47 @@
         <v>26</v>
       </c>
       <c r="N46" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="O46" s="1">
-        <v>8.9999999999999993E-3</v>
+        <v>0.18</v>
       </c>
       <c r="P46" s="1">
-        <v>0.09</v>
+        <v>0.36</v>
       </c>
       <c r="Q46" s="1">
-        <v>96583</v>
-      </c>
-    </row>
-    <row r="47" spans="1:17" x14ac:dyDescent="0.35">
+        <v>120740</v>
+      </c>
+    </row>
+    <row r="47" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A47" s="1"/>
       <c r="B47" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C47" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="D47" s="2" t="s">
         <v>275</v>
       </c>
-      <c r="D47" s="2" t="s">
+      <c r="E47" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F47" s="2" t="s">
         <v>276</v>
-      </c>
-      <c r="E47" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F47" s="2" t="s">
-        <v>277</v>
       </c>
       <c r="G47" s="1"/>
       <c r="H47" s="1">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I47" s="2" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="J47" s="2" t="s">
-        <v>252</v>
+        <v>23</v>
       </c>
       <c r="K47" s="2" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="L47" s="2" t="s">
         <v>25</v>
@@ -3919,47 +3908,47 @@
         <v>26</v>
       </c>
       <c r="N47" s="2" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="O47" s="1">
-        <v>0.17</v>
+        <v>2.4E-2</v>
       </c>
       <c r="P47" s="1">
-        <v>0.17</v>
+        <v>0.24</v>
       </c>
       <c r="Q47" s="1">
-        <v>20017</v>
-      </c>
-    </row>
-    <row r="48" spans="1:17" x14ac:dyDescent="0.35">
+        <v>44393</v>
+      </c>
+    </row>
+    <row r="48" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A48" s="1"/>
       <c r="B48" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C48" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="D48" s="2" t="s">
         <v>280</v>
       </c>
-      <c r="D48" s="2" t="s">
+      <c r="E48" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F48" s="2" t="s">
         <v>281</v>
-      </c>
-      <c r="E48" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F48" s="2" t="s">
-        <v>282</v>
       </c>
       <c r="G48" s="1"/>
       <c r="H48" s="1">
         <v>1</v>
       </c>
       <c r="I48" s="2" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="J48" s="2" t="s">
-        <v>226</v>
+        <v>256</v>
       </c>
       <c r="K48" s="2" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="L48" s="2" t="s">
         <v>25</v>
@@ -3968,47 +3957,47 @@
         <v>26</v>
       </c>
       <c r="N48" s="2" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="O48" s="1">
-        <v>0.1</v>
+        <v>0.18</v>
       </c>
       <c r="P48" s="1">
-        <v>0.1</v>
+        <v>0.18</v>
       </c>
       <c r="Q48" s="1">
-        <v>1845030</v>
-      </c>
-    </row>
-    <row r="49" spans="1:17" x14ac:dyDescent="0.35">
+        <v>51246</v>
+      </c>
+    </row>
+    <row r="49" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A49" s="1"/>
       <c r="B49" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C49" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="D49" s="2" t="s">
         <v>285</v>
       </c>
-      <c r="D49" s="2" t="s">
+      <c r="E49" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F49" s="2" t="s">
         <v>286</v>
-      </c>
-      <c r="E49" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F49" s="2" t="s">
-        <v>287</v>
       </c>
       <c r="G49" s="1"/>
       <c r="H49" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I49" s="2" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="J49" s="2" t="s">
-        <v>252</v>
+        <v>230</v>
       </c>
       <c r="K49" s="2" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="L49" s="2" t="s">
         <v>25</v>
@@ -4017,145 +4006,145 @@
         <v>26</v>
       </c>
       <c r="N49" s="2" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="O49" s="1">
-        <v>0.16</v>
+        <v>0.1</v>
       </c>
       <c r="P49" s="1">
-        <v>0.32</v>
+        <v>0.1</v>
       </c>
       <c r="Q49" s="1">
-        <v>22140</v>
-      </c>
-    </row>
-    <row r="50" spans="1:17" x14ac:dyDescent="0.35">
+        <v>1756024</v>
+      </c>
+    </row>
+    <row r="50" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A50" s="1"/>
       <c r="B50" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C50" s="2" t="s">
+        <v>289</v>
+      </c>
+      <c r="D50" s="2" t="s">
         <v>290</v>
       </c>
-      <c r="D50" s="2" t="s">
+      <c r="E50" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F50" s="2" t="s">
         <v>291</v>
-      </c>
-      <c r="E50" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F50" s="2" t="s">
-        <v>292</v>
       </c>
       <c r="G50" s="1"/>
       <c r="H50" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I50" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="J50" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="K50" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="L50" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M50" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="N50" s="2" t="s">
         <v>293</v>
       </c>
-      <c r="J50" s="2" t="s">
-        <v>294</v>
-      </c>
-      <c r="K50" s="2" t="s">
-        <v>295</v>
-      </c>
-      <c r="L50" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M50" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="N50" s="2" t="s">
-        <v>296</v>
-      </c>
       <c r="O50" s="1">
-        <v>0.72</v>
+        <v>0.17</v>
       </c>
       <c r="P50" s="1">
-        <v>0.72</v>
+        <v>0.34</v>
       </c>
       <c r="Q50" s="1">
-        <v>4220</v>
-      </c>
-    </row>
-    <row r="51" spans="1:17" x14ac:dyDescent="0.35">
+        <v>15278</v>
+      </c>
+    </row>
+    <row r="51" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A51" s="1"/>
       <c r="B51" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="E51" s="2" t="s">
         <v>20</v>
       </c>
       <c r="F51" s="2" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="G51" s="1"/>
       <c r="H51" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I51" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="J51" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="K51" s="2" t="s">
+        <v>299</v>
+      </c>
+      <c r="L51" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M51" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="N51" s="2" t="s">
         <v>300</v>
       </c>
-      <c r="J51" s="2" t="s">
-        <v>301</v>
-      </c>
-      <c r="K51" s="2" t="s">
-        <v>302</v>
-      </c>
-      <c r="L51" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M51" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="N51" s="2" t="s">
-        <v>303</v>
-      </c>
       <c r="O51" s="1">
-        <v>2.5</v>
+        <v>0.72</v>
       </c>
       <c r="P51" s="1">
-        <v>5</v>
+        <v>0.72</v>
       </c>
       <c r="Q51" s="1">
-        <v>6213</v>
-      </c>
-    </row>
-    <row r="52" spans="1:17" x14ac:dyDescent="0.35">
+        <v>1135</v>
+      </c>
+    </row>
+    <row r="52" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A52" s="1"/>
       <c r="B52" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="E52" s="2" t="s">
         <v>20</v>
       </c>
       <c r="F52" s="2" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="G52" s="1"/>
       <c r="H52" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I52" s="2" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="J52" s="2" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K52" s="2" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="L52" s="2" t="s">
         <v>25</v>
@@ -4164,129 +4153,129 @@
         <v>26</v>
       </c>
       <c r="N52" s="2" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="O52" s="1">
-        <v>0.26</v>
+        <v>2.48</v>
       </c>
       <c r="P52" s="1">
-        <v>0.26</v>
+        <v>4.96</v>
       </c>
       <c r="Q52" s="1">
-        <v>46240</v>
-      </c>
-    </row>
-    <row r="53" spans="1:17" x14ac:dyDescent="0.35">
+        <v>5688</v>
+      </c>
+    </row>
+    <row r="53" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A53" s="1"/>
       <c r="B53" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="E53" s="2" t="s">
         <v>20</v>
       </c>
       <c r="F53" s="2" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
       <c r="G53" s="1"/>
       <c r="H53" s="1">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="I53" s="2" t="s">
         <v>311</v>
       </c>
-      <c r="J53" s="1"/>
-      <c r="K53" s="1"/>
-      <c r="L53" s="1"/>
-      <c r="M53" s="1"/>
-      <c r="N53" s="1"/>
-      <c r="O53" s="1"/>
-      <c r="P53" s="1"/>
-      <c r="Q53" s="1"/>
-    </row>
-    <row r="54" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="J53" s="2" t="s">
+        <v>312</v>
+      </c>
+      <c r="K53" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="L53" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M53" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="N53" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="O53" s="1">
+        <v>0.26</v>
+      </c>
+      <c r="P53" s="1">
+        <v>0.26</v>
+      </c>
+      <c r="Q53" s="1">
+        <v>4779</v>
+      </c>
+    </row>
+    <row r="54" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A54" s="1"/>
       <c r="B54" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="E54" s="2" t="s">
         <v>20</v>
       </c>
       <c r="F54" s="2" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="G54" s="1"/>
       <c r="H54" s="1">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="I54" s="2" t="s">
-        <v>317</v>
-      </c>
-      <c r="J54" s="2" t="s">
-        <v>318</v>
-      </c>
-      <c r="K54" s="2" t="s">
-        <v>319</v>
-      </c>
-      <c r="L54" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M54" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="N54" s="2" t="s">
-        <v>320</v>
-      </c>
-      <c r="O54" s="1">
-        <v>2.41</v>
-      </c>
-      <c r="P54" s="1">
-        <v>2.41</v>
-      </c>
-      <c r="Q54" s="1">
-        <v>8840</v>
-      </c>
-    </row>
-    <row r="55" spans="1:17" x14ac:dyDescent="0.35">
+        <v>315</v>
+      </c>
+      <c r="J54" s="1"/>
+      <c r="K54" s="1"/>
+      <c r="L54" s="1"/>
+      <c r="M54" s="1"/>
+      <c r="N54" s="1"/>
+      <c r="O54" s="1"/>
+      <c r="P54" s="1"/>
+      <c r="Q54" s="1"/>
+    </row>
+    <row r="55" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A55" s="1"/>
       <c r="B55" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="E55" s="2" t="s">
         <v>20</v>
       </c>
       <c r="F55" s="2" t="s">
-        <v>323</v>
+        <v>320</v>
       </c>
       <c r="G55" s="1"/>
       <c r="H55" s="1">
         <v>1</v>
       </c>
       <c r="I55" s="2" t="s">
-        <v>324</v>
+        <v>321</v>
       </c>
       <c r="J55" s="2" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
       <c r="K55" s="2" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
       <c r="L55" s="2" t="s">
         <v>25</v>
@@ -4295,292 +4284,280 @@
         <v>26</v>
       </c>
       <c r="N55" s="2" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
       <c r="O55" s="1">
-        <v>7.18</v>
+        <v>2.41</v>
       </c>
       <c r="P55" s="1">
-        <v>7.18</v>
+        <v>2.41</v>
       </c>
       <c r="Q55" s="1">
-        <v>3741</v>
-      </c>
-    </row>
-    <row r="56" spans="1:17" x14ac:dyDescent="0.35">
+        <v>7734</v>
+      </c>
+    </row>
+    <row r="56" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A56" s="1"/>
       <c r="B56" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
       <c r="E56" s="2" t="s">
         <v>20</v>
       </c>
       <c r="F56" s="2" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
       <c r="G56" s="1"/>
       <c r="H56" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I56" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="J56" s="2" t="s">
+        <v>329</v>
+      </c>
+      <c r="K56" s="2" t="s">
+        <v>330</v>
+      </c>
+      <c r="L56" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M56" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="N56" s="2" t="s">
         <v>331</v>
       </c>
-      <c r="J56" s="2" t="s">
-        <v>325</v>
-      </c>
-      <c r="K56" s="2" t="s">
-        <v>328</v>
-      </c>
-      <c r="L56" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M56" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="N56" s="2" t="s">
-        <v>332</v>
-      </c>
       <c r="O56" s="1">
-        <v>10.35</v>
+        <v>8.15</v>
       </c>
       <c r="P56" s="1">
-        <v>20.7</v>
+        <v>8.15</v>
       </c>
       <c r="Q56" s="1">
-        <v>3848</v>
-      </c>
-    </row>
-    <row r="57" spans="1:17" x14ac:dyDescent="0.35">
+        <v>5241</v>
+      </c>
+    </row>
+    <row r="57" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A57" s="1"/>
       <c r="B57" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C57" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="D57" s="2" t="s">
         <v>333</v>
       </c>
-      <c r="D57" s="2" t="s">
+      <c r="E57" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F57" s="2" t="s">
         <v>334</v>
-      </c>
-      <c r="E57" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F57" s="2" t="s">
-        <v>335</v>
       </c>
       <c r="G57" s="1"/>
       <c r="H57" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I57" s="2" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="J57" s="2" t="s">
-        <v>115</v>
+        <v>329</v>
       </c>
       <c r="K57" s="2" t="s">
-        <v>337</v>
+        <v>332</v>
       </c>
       <c r="L57" s="2" t="s">
-        <v>338</v>
+        <v>25</v>
       </c>
       <c r="M57" s="2" t="s">
         <v>26</v>
       </c>
       <c r="N57" s="2" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
       <c r="O57" s="1">
-        <v>0.53</v>
+        <v>12.11</v>
       </c>
       <c r="P57" s="1">
-        <v>0.53</v>
+        <v>24.22</v>
       </c>
       <c r="Q57" s="1">
-        <v>8234</v>
-      </c>
-    </row>
-    <row r="58" spans="1:17" x14ac:dyDescent="0.35">
+        <v>1685</v>
+      </c>
+    </row>
+    <row r="58" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A58" s="1"/>
       <c r="B58" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
       <c r="E58" s="2" t="s">
         <v>20</v>
       </c>
       <c r="F58" s="2" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
       <c r="G58" s="1"/>
       <c r="H58" s="1">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I58" s="2" t="s">
-        <v>343</v>
+        <v>340</v>
       </c>
       <c r="J58" s="2" t="s">
-        <v>344</v>
+        <v>114</v>
       </c>
       <c r="K58" s="2" t="s">
-        <v>345</v>
+        <v>341</v>
       </c>
       <c r="L58" s="2" t="s">
-        <v>25</v>
+        <v>342</v>
       </c>
       <c r="M58" s="2" t="s">
         <v>26</v>
       </c>
       <c r="N58" s="2" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="O58" s="1">
-        <v>1.33</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="P58" s="1">
-        <v>5.32</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="Q58" s="1">
-        <v>40986</v>
-      </c>
-    </row>
-    <row r="59" spans="1:17" x14ac:dyDescent="0.35">
+        <v>7454</v>
+      </c>
+    </row>
+    <row r="59" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A59" s="1"/>
       <c r="B59" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>347</v>
+        <v>344</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="E59" s="2" t="s">
         <v>20</v>
       </c>
       <c r="F59" s="2" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="G59" s="1"/>
       <c r="H59" s="1">
         <v>1</v>
       </c>
       <c r="I59" s="2" t="s">
+        <v>344</v>
+      </c>
+      <c r="J59" s="2" t="s">
         <v>347</v>
       </c>
-      <c r="J59" s="2" t="s">
-        <v>350</v>
-      </c>
       <c r="K59" s="2" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="L59" s="2" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="M59" s="2" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="N59" s="2" t="s">
-        <v>352</v>
-      </c>
-      <c r="O59" s="1">
-        <v>12.95</v>
-      </c>
-      <c r="P59" s="1">
-        <v>12.95</v>
-      </c>
-      <c r="Q59" s="1">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="60" spans="1:17" x14ac:dyDescent="0.35">
+        <v>349</v>
+      </c>
+      <c r="O59" s="1"/>
+      <c r="P59" s="1"/>
+      <c r="Q59" s="1"/>
+    </row>
+    <row r="60" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A60" s="1"/>
       <c r="B60" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
       <c r="E60" s="2" t="s">
         <v>20</v>
       </c>
       <c r="F60" s="2" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
       <c r="G60" s="1"/>
       <c r="H60" s="1">
         <v>1</v>
       </c>
       <c r="I60" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="J60" s="2" t="s">
+        <v>347</v>
+      </c>
+      <c r="K60" s="2" t="s">
         <v>353</v>
       </c>
-      <c r="J60" s="2" t="s">
-        <v>350</v>
-      </c>
-      <c r="K60" s="2" t="s">
-        <v>356</v>
-      </c>
       <c r="L60" s="2" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="M60" s="2" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="N60" s="2" t="s">
-        <v>357</v>
-      </c>
-      <c r="O60" s="1">
-        <v>12.5</v>
-      </c>
-      <c r="P60" s="1">
-        <v>12.5</v>
-      </c>
-      <c r="Q60" s="1">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="61" spans="1:17" x14ac:dyDescent="0.35">
+        <v>354</v>
+      </c>
+      <c r="O60" s="1"/>
+      <c r="P60" s="1"/>
+      <c r="Q60" s="1"/>
+    </row>
+    <row r="61" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A61" s="1"/>
       <c r="B61" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>358</v>
+        <v>355</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>359</v>
+        <v>356</v>
       </c>
       <c r="E61" s="2" t="s">
         <v>20</v>
       </c>
       <c r="F61" s="2" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
       <c r="G61" s="1"/>
       <c r="H61" s="1">
         <v>1</v>
       </c>
       <c r="I61" s="2" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
       <c r="J61" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="K61" s="2" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="L61" s="2" t="s">
         <v>25</v>
@@ -4589,7 +4566,7 @@
         <v>26</v>
       </c>
       <c r="N61" s="2" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="O61" s="1">
         <v>0.52</v>
@@ -4598,38 +4575,38 @@
         <v>0.52</v>
       </c>
       <c r="Q61" s="1">
-        <v>11089</v>
-      </c>
-    </row>
-    <row r="62" spans="1:17" x14ac:dyDescent="0.35">
+        <v>5003</v>
+      </c>
+    </row>
+    <row r="62" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A62" s="1"/>
       <c r="B62" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="E62" s="2" t="s">
         <v>20</v>
       </c>
       <c r="F62" s="2" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="G62" s="1"/>
       <c r="H62" s="1">
         <v>1</v>
       </c>
       <c r="I62" s="2" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="J62" s="2" t="s">
-        <v>301</v>
+        <v>305</v>
       </c>
       <c r="K62" s="2" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="L62" s="2" t="s">
         <v>25</v>
@@ -4638,56 +4615,56 @@
         <v>26</v>
       </c>
       <c r="N62" s="2" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="O62" s="1">
-        <v>2.42</v>
+        <v>2.4</v>
       </c>
       <c r="P62" s="1">
-        <v>2.42</v>
+        <v>2.4</v>
       </c>
       <c r="Q62" s="1">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="63" spans="1:17" x14ac:dyDescent="0.35">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="63" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A63" s="1"/>
       <c r="B63" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="E63" s="2" t="s">
         <v>20</v>
       </c>
       <c r="F63" s="2" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
       <c r="G63" s="1"/>
       <c r="H63" s="1">
         <v>1</v>
       </c>
       <c r="I63" s="2" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="J63" s="2" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="K63" s="2" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
       <c r="L63" s="2" t="s">
         <v>25</v>
       </c>
       <c r="M63" s="2" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="N63" s="2" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
       <c r="O63" s="1">
         <v>2.0699999999999998</v>
@@ -4696,38 +4673,38 @@
         <v>2.0699999999999998</v>
       </c>
       <c r="Q63" s="1">
-        <v>2068</v>
-      </c>
-    </row>
-    <row r="64" spans="1:17" x14ac:dyDescent="0.35">
+        <v>766</v>
+      </c>
+    </row>
+    <row r="64" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A64" s="1"/>
       <c r="B64" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>377</v>
+        <v>374</v>
       </c>
       <c r="E64" s="2" t="s">
         <v>20</v>
       </c>
       <c r="F64" s="2" t="s">
-        <v>378</v>
+        <v>375</v>
       </c>
       <c r="G64" s="1"/>
       <c r="H64" s="1">
         <v>1</v>
       </c>
       <c r="I64" s="2" t="s">
-        <v>379</v>
+        <v>376</v>
       </c>
       <c r="J64" s="2" t="s">
-        <v>380</v>
+        <v>377</v>
       </c>
       <c r="K64" s="2" t="s">
-        <v>381</v>
+        <v>378</v>
       </c>
       <c r="L64" s="2" t="s">
         <v>25</v>
@@ -4736,7 +4713,7 @@
         <v>26</v>
       </c>
       <c r="N64" s="2" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
       <c r="O64" s="1">
         <v>0.42</v>
@@ -4745,38 +4722,38 @@
         <v>0.42</v>
       </c>
       <c r="Q64" s="1">
-        <v>219752</v>
-      </c>
-    </row>
-    <row r="65" spans="1:17" x14ac:dyDescent="0.35">
+        <v>222737</v>
+      </c>
+    </row>
+    <row r="65" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A65" s="1"/>
       <c r="B65" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
       <c r="E65" s="2" t="s">
         <v>20</v>
       </c>
       <c r="F65" s="2" t="s">
-        <v>384</v>
+        <v>381</v>
       </c>
       <c r="G65" s="1"/>
       <c r="H65" s="1">
         <v>1</v>
       </c>
       <c r="I65" s="2" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="J65" s="2" t="s">
-        <v>386</v>
+        <v>383</v>
       </c>
       <c r="K65" s="2" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
       <c r="L65" s="2" t="s">
         <v>25</v>
@@ -4785,16 +4762,16 @@
         <v>26</v>
       </c>
       <c r="N65" s="2" t="s">
-        <v>388</v>
+        <v>385</v>
       </c>
       <c r="O65" s="1">
-        <v>0.56999999999999995</v>
+        <v>0.62</v>
       </c>
       <c r="P65" s="1">
-        <v>0.56999999999999995</v>
+        <v>0.62</v>
       </c>
       <c r="Q65" s="1">
-        <v>6066</v>
+        <v>9013</v>
       </c>
     </row>
   </sheetData>

</xml_diff>